<commit_message>
Add few more common words
</commit_message>
<xml_diff>
--- a/Aakhar_list.xlsx
+++ b/Aakhar_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/prithvirajnarendra/Documents/Aakhar App/Aakhar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB148D1C-56CB-B84D-BE07-1FAFD96384E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24C0F5BC-CB96-A944-A283-9B62FEEBDFB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10520" yWindow="-28200" windowWidth="51200" windowHeight="28200" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Common Words" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="938" uniqueCount="742">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="765">
   <si>
     <t>Hindi</t>
   </si>
@@ -2255,6 +2255,75 @@
   </si>
   <si>
     <t>Our language is our identity</t>
+  </si>
+  <si>
+    <t>Ink</t>
+  </si>
+  <si>
+    <t>Inkpot</t>
+  </si>
+  <si>
+    <t>Instant</t>
+  </si>
+  <si>
+    <t>Jackal</t>
+  </si>
+  <si>
+    <t>King</t>
+  </si>
+  <si>
+    <t>Own</t>
+  </si>
+  <si>
+    <t>Out</t>
+  </si>
+  <si>
+    <t>Queen</t>
+  </si>
+  <si>
+    <t>Quality</t>
+  </si>
+  <si>
+    <t>Xray</t>
+  </si>
+  <si>
+    <t>Zebra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">स्याही </t>
+  </si>
+  <si>
+    <t xml:space="preserve">दवात </t>
+  </si>
+  <si>
+    <t xml:space="preserve">तुरंत </t>
+  </si>
+  <si>
+    <t>गीदड़/ शियार</t>
+  </si>
+  <si>
+    <t xml:space="preserve">राजा </t>
+  </si>
+  <si>
+    <t xml:space="preserve">पतंग </t>
+  </si>
+  <si>
+    <t xml:space="preserve">अपना </t>
+  </si>
+  <si>
+    <t xml:space="preserve">बाहिर </t>
+  </si>
+  <si>
+    <t xml:space="preserve">रानी </t>
+  </si>
+  <si>
+    <t xml:space="preserve">दर्जा/ स्तर </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ऐक्स- रे </t>
+  </si>
+  <si>
+    <t xml:space="preserve">जेब्रा </t>
   </si>
 </sst>
 </file>
@@ -4027,32 +4096,224 @@
         <v>692</v>
       </c>
     </row>
-    <row r="87" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="88" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="89" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="90" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="91" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="92" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="93" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="94" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="95" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="96" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="100" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="101" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="102" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="103" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="104" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="105" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="106" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="107" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="108" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="109" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="110" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="111" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="112" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="87" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A87" t="s">
+        <v>753</v>
+      </c>
+      <c r="B87" t="s">
+        <v>742</v>
+      </c>
+      <c r="C87" t="s">
+        <v>753</v>
+      </c>
+      <c r="D87" t="s">
+        <v>753</v>
+      </c>
+      <c r="E87" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A88" t="s">
+        <v>754</v>
+      </c>
+      <c r="B88" t="s">
+        <v>743</v>
+      </c>
+      <c r="C88" t="s">
+        <v>754</v>
+      </c>
+      <c r="D88" t="s">
+        <v>754</v>
+      </c>
+      <c r="E88" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A89" t="s">
+        <v>755</v>
+      </c>
+      <c r="B89" t="s">
+        <v>744</v>
+      </c>
+      <c r="C89" t="s">
+        <v>755</v>
+      </c>
+      <c r="D89" t="s">
+        <v>755</v>
+      </c>
+      <c r="E89" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A90" t="s">
+        <v>756</v>
+      </c>
+      <c r="B90" t="s">
+        <v>745</v>
+      </c>
+      <c r="C90" t="s">
+        <v>756</v>
+      </c>
+      <c r="D90" t="s">
+        <v>756</v>
+      </c>
+      <c r="E90" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A91" t="s">
+        <v>757</v>
+      </c>
+      <c r="B91" t="s">
+        <v>746</v>
+      </c>
+      <c r="C91" t="s">
+        <v>757</v>
+      </c>
+      <c r="D91" t="s">
+        <v>757</v>
+      </c>
+      <c r="E91" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A92" t="s">
+        <v>758</v>
+      </c>
+      <c r="B92" t="s">
+        <v>575</v>
+      </c>
+      <c r="C92" t="s">
+        <v>758</v>
+      </c>
+      <c r="D92" t="s">
+        <v>758</v>
+      </c>
+      <c r="E92" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A93" t="s">
+        <v>759</v>
+      </c>
+      <c r="B93" t="s">
+        <v>747</v>
+      </c>
+      <c r="C93" t="s">
+        <v>759</v>
+      </c>
+      <c r="D93" t="s">
+        <v>759</v>
+      </c>
+      <c r="E93" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A94" t="s">
+        <v>760</v>
+      </c>
+      <c r="B94" t="s">
+        <v>748</v>
+      </c>
+      <c r="C94" t="s">
+        <v>760</v>
+      </c>
+      <c r="D94" t="s">
+        <v>760</v>
+      </c>
+      <c r="E94" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A95" t="s">
+        <v>761</v>
+      </c>
+      <c r="B95" t="s">
+        <v>749</v>
+      </c>
+      <c r="C95" t="s">
+        <v>761</v>
+      </c>
+      <c r="D95" t="s">
+        <v>761</v>
+      </c>
+      <c r="E95" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A96" t="s">
+        <v>762</v>
+      </c>
+      <c r="B96" t="s">
+        <v>750</v>
+      </c>
+      <c r="C96" t="s">
+        <v>762</v>
+      </c>
+      <c r="D96" t="s">
+        <v>762</v>
+      </c>
+      <c r="E96" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A97" t="s">
+        <v>763</v>
+      </c>
+      <c r="B97" t="s">
+        <v>751</v>
+      </c>
+      <c r="C97" t="s">
+        <v>763</v>
+      </c>
+      <c r="D97" t="s">
+        <v>763</v>
+      </c>
+      <c r="E97" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A98" t="s">
+        <v>764</v>
+      </c>
+      <c r="B98" t="s">
+        <v>752</v>
+      </c>
+      <c r="C98" t="s">
+        <v>764</v>
+      </c>
+      <c r="D98" t="s">
+        <v>764</v>
+      </c>
+      <c r="E98" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="100" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="101" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="102" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="103" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="104" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="105" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="106" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="107" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="108" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="109" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="110" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="111" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="112" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="113" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="114" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="115" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>

</xml_diff>